<commit_message>
WhiteBoard Update - 2026-04-30 09:05:19
</commit_message>
<xml_diff>
--- a/MyPreply/PreplyAnalyse-2.xlsx
+++ b/MyPreply/PreplyAnalyse-2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Berechnung" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="43">
   <si>
     <t xml:space="preserve">h/Tag</t>
   </si>
@@ -51,7 +51,13 @@
     <t xml:space="preserve">23 → 16,5 → 20</t>
   </si>
   <si>
+    <t xml:space="preserve">15 → 17</t>
+  </si>
+  <si>
     <t xml:space="preserve">Profil geändert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verfügbarkeit</t>
   </si>
   <si>
     <t xml:space="preserve">Hoped +</t>
@@ -2750,6 +2756,12 @@
       <c r="AG2" s="2" t="n">
         <v>1721</v>
       </c>
+      <c r="AH2" s="2" t="n">
+        <v>1768</v>
+      </c>
+      <c r="AI2" s="2" t="n">
+        <v>1865</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
@@ -2800,6 +2812,12 @@
       <c r="AG3" s="17" t="n">
         <v>271</v>
       </c>
+      <c r="AH3" s="2" t="n">
+        <v>177</v>
+      </c>
+      <c r="AI3" s="2" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G4" s="2" t="s">
@@ -2823,16 +2841,22 @@
       <c r="AG4" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="AH4" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="AC5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="AH5" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18"/>
       <c r="B11" s="18" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C11" s="18" t="n">
         <v>3</v>
@@ -2984,7 +3008,7 @@
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21"/>
       <c r="B14" s="21" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C14" s="21"/>
       <c r="D14" s="21"/>
@@ -3308,7 +3332,7 @@
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21"/>
       <c r="B18" s="21" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C18" s="28"/>
       <c r="D18" s="28"/>
@@ -3387,7 +3411,7 @@
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="21"/>
       <c r="B19" s="21" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C19" s="26"/>
       <c r="D19" s="26"/>
@@ -3466,7 +3490,7 @@
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="21"/>
       <c r="B20" s="21" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C20" s="28"/>
       <c r="D20" s="28"/>
@@ -3545,7 +3569,7 @@
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="21"/>
       <c r="B21" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C21" s="26"/>
       <c r="D21" s="26"/>
@@ -3625,7 +3649,7 @@
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23"/>
       <c r="B23" s="31" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3633,7 +3657,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C24" s="32" t="n">
         <v>15</v>
@@ -3711,7 +3735,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C26" s="32" t="n">
         <v>15</v>
@@ -3789,7 +3813,7 @@
         <v>3</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C28" s="32" t="n">
         <v>15</v>
@@ -3856,7 +3880,7 @@
       <c r="M29" s="18"/>
       <c r="N29" s="18"/>
       <c r="O29" s="36" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="P29" s="18"/>
       <c r="Q29" s="18"/>
@@ -3869,7 +3893,7 @@
         <v>4</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C30" s="32" t="n">
         <v>23</v>
@@ -3937,7 +3961,7 @@
       <c r="N31" s="18"/>
       <c r="O31" s="18"/>
       <c r="P31" s="18" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="Q31" s="18"/>
       <c r="R31" s="18"/>
@@ -3949,7 +3973,7 @@
         <v>5</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C32" s="32" t="n">
         <v>15</v>
@@ -4027,7 +4051,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C34" s="32" t="n">
         <v>18</v>
@@ -4105,7 +4129,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C36" s="32" t="n">
         <v>14</v>
@@ -4170,7 +4194,7 @@
       <c r="K37" s="18"/>
       <c r="L37" s="18"/>
       <c r="M37" s="18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="N37" s="18"/>
       <c r="O37" s="18"/>
@@ -4185,7 +4209,7 @@
         <v>8</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C38" s="32" t="n">
         <v>18</v>
@@ -4263,7 +4287,7 @@
         <v>9</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C40" s="32" t="n">
         <v>12</v>
@@ -4328,7 +4352,7 @@
       <c r="K41" s="18"/>
       <c r="L41" s="18"/>
       <c r="M41" s="18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="N41" s="18"/>
       <c r="O41" s="18"/>
@@ -4343,7 +4367,7 @@
         <v>10</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C42" s="32" t="n">
         <v>15</v>
@@ -4412,16 +4436,16 @@
       <c r="O43" s="18"/>
       <c r="P43" s="18"/>
       <c r="Q43" s="18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="R43" s="18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="S43" s="18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="T43" s="18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4429,7 +4453,7 @@
         <v>11</v>
       </c>
       <c r="B44" s="21" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C44" s="32" t="n">
         <v>15</v>
@@ -4507,7 +4531,7 @@
         <v>12</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C46" s="32" t="n">
         <v>15</v>
@@ -4585,7 +4609,7 @@
         <v>13</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C48" s="32" t="n">
         <v>19</v>
@@ -4663,7 +4687,7 @@
         <v>14</v>
       </c>
       <c r="B50" s="39" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C50" s="40" t="n">
         <v>21</v>
@@ -4682,21 +4706,21 @@
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D51" s="42"/>
       <c r="E51" s="42"/>
       <c r="J51" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="R51" s="43" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="S51" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="U51" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4706,7 +4730,7 @@
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="18"/>
       <c r="B53" s="18" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C53" s="18" t="n">
         <v>10</v>
@@ -4798,7 +4822,7 @@
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="21"/>
       <c r="B56" s="21" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C56" s="21"/>
       <c r="D56" s="21"/>
@@ -4942,7 +4966,7 @@
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="21"/>
       <c r="B58" s="21" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C58" s="28"/>
       <c r="D58" s="28"/>
@@ -5079,7 +5103,7 @@
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="21"/>
       <c r="B59" s="21" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C59" s="26"/>
       <c r="D59" s="26"/>
@@ -5216,7 +5240,7 @@
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="21"/>
       <c r="B60" s="21" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C60" s="28"/>
       <c r="D60" s="28"/>
@@ -5353,7 +5377,7 @@
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="21"/>
       <c r="B61" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C61" s="26"/>
       <c r="D61" s="26"/>
@@ -5529,7 +5553,7 @@
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="23"/>
       <c r="B63" s="31" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F63" s="2"/>
       <c r="AK63" s="2"/>
@@ -5539,7 +5563,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="21" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C64" s="32" t="n">
         <v>15</v>
@@ -5654,7 +5678,7 @@
         <v>2</v>
       </c>
       <c r="B65" s="21" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C65" s="32" t="n">
         <v>15</v>
@@ -5769,7 +5793,7 @@
         <v>3</v>
       </c>
       <c r="B66" s="21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C66" s="32" t="n">
         <v>15</v>
@@ -5884,7 +5908,7 @@
         <v>4</v>
       </c>
       <c r="B67" s="21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C67" s="32" t="n">
         <v>23</v>
@@ -5935,7 +5959,7 @@
         <v>5</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C68" s="32" t="n">
         <v>15</v>
@@ -6050,7 +6074,7 @@
         <v>6</v>
       </c>
       <c r="B69" s="21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C69" s="32" t="n">
         <v>18</v>
@@ -6165,7 +6189,7 @@
         <v>7</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C70" s="32" t="n">
         <v>14</v>
@@ -6280,7 +6304,7 @@
         <v>8</v>
       </c>
       <c r="B71" s="21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C71" s="32" t="n">
         <v>18</v>
@@ -6395,7 +6419,7 @@
         <v>9</v>
       </c>
       <c r="B72" s="21" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C72" s="32" t="n">
         <v>18</v>
@@ -6510,7 +6534,7 @@
         <v>10</v>
       </c>
       <c r="B73" s="21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C73" s="32" t="n">
         <v>15</v>
@@ -6625,7 +6649,7 @@
         <v>11</v>
       </c>
       <c r="B74" s="21" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C74" s="32" t="n">
         <v>15</v>
@@ -6740,7 +6764,7 @@
         <v>12</v>
       </c>
       <c r="B75" s="21" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C75" s="32" t="n">
         <v>15</v>
@@ -6855,7 +6879,7 @@
         <v>13</v>
       </c>
       <c r="B76" s="21" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C76" s="32" t="n">
         <v>19</v>
@@ -6970,7 +6994,7 @@
         <v>14</v>
       </c>
       <c r="B77" s="39" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C77" s="44" t="n">
         <v>21</v>
@@ -7085,7 +7109,7 @@
         <v>14</v>
       </c>
       <c r="B78" s="39" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C78" s="44" t="n">
         <v>21</v>
@@ -7200,7 +7224,7 @@
         <v>15</v>
       </c>
       <c r="B79" s="39" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C79" s="44" t="n">
         <v>21</v>
@@ -7315,7 +7339,7 @@
         <v>15</v>
       </c>
       <c r="B80" s="39" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C80" s="44" t="n">
         <v>21</v>
@@ -7473,7 +7497,7 @@
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18"/>
       <c r="B4" s="18" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="18" t="n">
         <v>10</v>
@@ -7703,7 +7727,7 @@
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21"/>
       <c r="B9" s="21" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C9" s="28"/>
       <c r="D9" s="28"/>
@@ -7747,7 +7771,7 @@
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21"/>
       <c r="B10" s="21" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -7791,7 +7815,7 @@
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21"/>
       <c r="B11" s="21" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C11" s="28"/>
       <c r="D11" s="28"/>
@@ -7835,7 +7859,7 @@
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21"/>
       <c r="B12" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C12" s="26"/>
       <c r="D12" s="26"/>
@@ -7918,7 +7942,7 @@
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23"/>
       <c r="B14" s="31" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7926,7 +7950,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C15" s="32" t="n">
         <v>15</v>
@@ -7950,7 +7974,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C16" s="32" t="n">
         <v>15</v>
@@ -7974,7 +7998,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C17" s="32" t="n">
         <v>15</v>
@@ -7998,7 +8022,7 @@
         <v>4</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C18" s="32" t="n">
         <v>23</v>
@@ -8020,7 +8044,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C19" s="32" t="n">
         <v>15</v>
@@ -8044,7 +8068,7 @@
         <v>6</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C20" s="32" t="n">
         <v>18</v>
@@ -8068,7 +8092,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C21" s="32" t="n">
         <v>14</v>
@@ -8092,7 +8116,7 @@
         <v>8</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C22" s="32" t="n">
         <v>18</v>
@@ -8116,7 +8140,7 @@
         <v>9</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C23" s="32" t="n">
         <v>18</v>
@@ -8140,7 +8164,7 @@
         <v>10</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C24" s="32" t="n">
         <v>15</v>
@@ -8164,7 +8188,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C25" s="32" t="n">
         <v>15</v>
@@ -8188,7 +8212,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C26" s="32" t="n">
         <v>15</v>
@@ -8212,7 +8236,7 @@
         <v>13</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C27" s="32" t="n">
         <v>19</v>
@@ -8236,7 +8260,7 @@
         <v>14</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C28" s="40" t="n">
         <v>21</v>

</xml_diff>

<commit_message>
WhiteBoard Update - 2026-05-02 09:07:04
</commit_message>
<xml_diff>
--- a/MyPreply/PreplyAnalyse-2.xlsx
+++ b/MyPreply/PreplyAnalyse-2.xlsx
@@ -355,7 +355,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -538,6 +538,10 @@
     </xf>
     <xf numFmtId="166" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -727,7 +731,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B6:W56"/>
+  <dimension ref="B6:W60"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.53"/>
@@ -3228,6 +3232,78 @@
       <c r="F56" s="6" t="n">
         <f aca="false">D56/1.18</f>
         <v>16.6779661016949</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C57" s="3" t="n">
+        <f aca="false">C56+$B$6</f>
+        <v>24.25</v>
+      </c>
+      <c r="D57" s="4" t="n">
+        <f aca="false">C57-(C57*0.18)</f>
+        <v>19.885</v>
+      </c>
+      <c r="E57" s="5" t="n">
+        <f aca="false">C57/1.18</f>
+        <v>20.5508474576271</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <f aca="false">D57/1.18</f>
+        <v>16.8516949152542</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C58" s="3" t="n">
+        <f aca="false">C57+$B$6</f>
+        <v>24.5</v>
+      </c>
+      <c r="D58" s="4" t="n">
+        <f aca="false">C58-(C58*0.18)</f>
+        <v>20.09</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <f aca="false">C58/1.18</f>
+        <v>20.7627118644068</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <f aca="false">D58/1.18</f>
+        <v>17.0254237288136</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C59" s="3" t="n">
+        <f aca="false">C58+$B$6</f>
+        <v>24.75</v>
+      </c>
+      <c r="D59" s="4" t="n">
+        <f aca="false">C59-(C59*0.18)</f>
+        <v>20.295</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <f aca="false">C59/1.18</f>
+        <v>20.9745762711864</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <f aca="false">D59/1.18</f>
+        <v>17.1991525423729</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C60" s="3" t="n">
+        <f aca="false">C59+$B$6</f>
+        <v>25</v>
+      </c>
+      <c r="D60" s="4" t="n">
+        <f aca="false">C60-(C60*0.18)</f>
+        <v>20.5</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <f aca="false">C60/1.18</f>
+        <v>21.1864406779661</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <f aca="false">D60/1.18</f>
+        <v>17.3728813559322</v>
       </c>
     </row>
   </sheetData>
@@ -8028,10 +8104,11 @@
       <c r="B1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" s="0"/>
+      <c r="F1" s="1" t="n">
         <v>83</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="G1" s="1" t="n">
         <v>91</v>
       </c>
     </row>
@@ -8039,37 +8116,44 @@
       <c r="B2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="1" t="n">
-        <v>1865</v>
-      </c>
+      <c r="E2" s="0"/>
       <c r="F2" s="1" t="n">
         <v>1865</v>
       </c>
+      <c r="G2" s="1" t="n">
+        <v>1865</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="0"/>
+      <c r="F3" s="1" t="n">
         <v>65</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="G3" s="1" t="n">
         <v>68</v>
+      </c>
+      <c r="H3" s="46" t="n">
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="0"/>
+      <c r="F4" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="F4" s="46" t="s">
+      <c r="G4" s="47" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F5" s="1" t="s">
+      <c r="E5" s="0"/>
+      <c r="G5" s="1" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WhiteBoard Update - 2026-05-04 09:14:06
</commit_message>
<xml_diff>
--- a/MyPreply/PreplyAnalyse-2.xlsx
+++ b/MyPreply/PreplyAnalyse-2.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="57">
   <si>
     <t xml:space="preserve">Kenny kündigt Abbo</t>
   </si>
@@ -34,10 +34,16 @@
     <t xml:space="preserve">Position</t>
   </si>
   <si>
+    <t xml:space="preserve">zeit umstellung</t>
+  </si>
+  <si>
     <t xml:space="preserve">Price</t>
   </si>
   <si>
     <t xml:space="preserve">25 - &gt; 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 → 25</t>
   </si>
   <si>
     <t xml:space="preserve">CheckTime</t>
@@ -47,9 +53,6 @@
   </si>
   <si>
     <t xml:space="preserve">Visitors 7 d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zeitfenster</t>
   </si>
   <si>
     <t xml:space="preserve">h/Tag</t>
@@ -197,7 +200,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="166" formatCode="hh:mm:ss"/>
@@ -205,7 +208,6 @@
     <numFmt numFmtId="168" formatCode="#,##0.00\ [$€-407];[RED]\-#,##0.00\ [$€-407]"/>
     <numFmt numFmtId="169" formatCode="[$-407]General"/>
     <numFmt numFmtId="170" formatCode="[$$-409]#,##0;[RED]\-[$$-409]#,##0"/>
-    <numFmt numFmtId="171" formatCode="dd/mm/yy"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -393,11 +395,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -405,24 +411,20 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -557,7 +559,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -788,109 +790,128 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:E9"/>
+  <dimension ref="A2:F9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26.05"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2" t="n">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="3" t="n">
         <v>46144</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>46145</v>
       </c>
+      <c r="F3" s="3" t="n">
+        <v>46146</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>86</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="4" t="n">
         <v>246</v>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="2" t="n">
         <v>246</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>426</v>
       </c>
+      <c r="F4" s="0" t="n">
+        <v>186</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="5" t="n">
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="5" t="n">
+        <v>0.352083333333333</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="6" t="n">
+      <c r="F6" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="8" t="n">
         <v>0.882638888888889</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E7" s="6" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="7" t="n">
+      <c r="F7" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="n">
         <v>1865</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D8" s="2" t="n">
         <v>1971</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>1971</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1" t="n">
+      <c r="F8" s="0" t="n">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="n">
         <v>371</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
+      <c r="F9" s="0" t="n">
+        <v>59</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -911,86 +932,86 @@
   <dimension ref="B6:W60"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="8" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="12" style="8" width="14.6"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="12" style="1" width="14.6"/>
   </cols>
   <sheetData>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="n">
         <v>0.25</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="M6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="N6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="O6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="R6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="S6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="T6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="U6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="V6" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="W6" s="8" t="s">
-        <v>9</v>
+      <c r="J6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="W6" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="K7" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="L7" s="8" t="n">
+      <c r="L7" s="1" t="n">
         <v>3.5</v>
       </c>
-      <c r="M7" s="8" t="n">
+      <c r="M7" s="1" t="n">
         <v>3.7</v>
       </c>
-      <c r="N7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="O7" s="8" t="n">
+      <c r="N7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" s="1" t="n">
         <v>4.5</v>
       </c>
-      <c r="R7" s="8" t="n">
+      <c r="R7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="S7" s="8" t="n">
+      <c r="S7" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="T7" s="8" t="n">
+      <c r="T7" s="1" t="n">
         <v>3.5</v>
       </c>
-      <c r="U7" s="8" t="n">
+      <c r="U7" s="1" t="n">
         <v>3.7</v>
       </c>
-      <c r="V7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="W7" s="8" t="n">
+      <c r="V7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="W7" s="1" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -1709,19 +1730,19 @@
       <c r="I19" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="1" t="n">
         <f aca="false">J9*20</f>
         <v>426.4</v>
       </c>
-      <c r="K19" s="8" t="n">
+      <c r="K19" s="1" t="n">
         <f aca="false">K9*20</f>
         <v>639.6</v>
       </c>
-      <c r="L19" s="8" t="n">
+      <c r="L19" s="1" t="n">
         <f aca="false">L9*20</f>
         <v>746.2</v>
       </c>
-      <c r="M19" s="8" t="n">
+      <c r="M19" s="1" t="n">
         <f aca="false">M9*20</f>
         <v>788.84</v>
       </c>
@@ -1782,19 +1803,19 @@
       <c r="I20" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="J20" s="1" t="n">
         <f aca="false">J10*20</f>
         <v>459.2</v>
       </c>
-      <c r="K20" s="8" t="n">
+      <c r="K20" s="1" t="n">
         <f aca="false">K10*20</f>
         <v>688.8</v>
       </c>
-      <c r="L20" s="8" t="n">
+      <c r="L20" s="1" t="n">
         <f aca="false">L10*20</f>
         <v>803.6</v>
       </c>
-      <c r="M20" s="8" t="n">
+      <c r="M20" s="1" t="n">
         <f aca="false">M10*20</f>
         <v>849.52</v>
       </c>
@@ -1858,19 +1879,19 @@
       <c r="I21" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="J21" s="8" t="n">
+      <c r="J21" s="1" t="n">
         <f aca="false">J11*20</f>
         <v>492</v>
       </c>
-      <c r="K21" s="8" t="n">
+      <c r="K21" s="1" t="n">
         <f aca="false">K11*20</f>
         <v>738</v>
       </c>
-      <c r="L21" s="8" t="n">
+      <c r="L21" s="1" t="n">
         <f aca="false">L11*20</f>
         <v>861</v>
       </c>
-      <c r="M21" s="8" t="n">
+      <c r="M21" s="1" t="n">
         <f aca="false">M11*20</f>
         <v>910.2</v>
       </c>
@@ -1931,19 +1952,19 @@
       <c r="I22" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="J22" s="8" t="n">
+      <c r="J22" s="1" t="n">
         <f aca="false">$J12*20</f>
         <v>524.8</v>
       </c>
-      <c r="K22" s="8" t="n">
+      <c r="K22" s="1" t="n">
         <f aca="false">$K$12*20</f>
         <v>787.2</v>
       </c>
-      <c r="L22" s="8" t="n">
+      <c r="L22" s="1" t="n">
         <f aca="false">$L$12*20</f>
         <v>918.4</v>
       </c>
-      <c r="M22" s="8" t="n">
+      <c r="M22" s="1" t="n">
         <f aca="false">$M$12*20</f>
         <v>970.88</v>
       </c>
@@ -2004,19 +2025,19 @@
       <c r="I23" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J23" s="8" t="n">
+      <c r="J23" s="1" t="n">
         <f aca="false">$J13*20</f>
         <v>557.6</v>
       </c>
-      <c r="K23" s="8" t="n">
+      <c r="K23" s="1" t="n">
         <f aca="false">$K$13*20</f>
         <v>836.4</v>
       </c>
-      <c r="L23" s="8" t="n">
+      <c r="L23" s="1" t="n">
         <f aca="false">$L$13*20</f>
         <v>975.8</v>
       </c>
-      <c r="M23" s="8" t="n">
+      <c r="M23" s="1" t="n">
         <f aca="false">$M$13*20</f>
         <v>1031.56</v>
       </c>
@@ -2077,19 +2098,19 @@
       <c r="I24" s="19" t="n">
         <v>18</v>
       </c>
-      <c r="J24" s="8" t="n">
+      <c r="J24" s="1" t="n">
         <f aca="false">$J14*20</f>
         <v>590.4</v>
       </c>
-      <c r="K24" s="8" t="n">
+      <c r="K24" s="1" t="n">
         <f aca="false">$K$14*20</f>
         <v>885.6</v>
       </c>
-      <c r="L24" s="8" t="n">
+      <c r="L24" s="1" t="n">
         <f aca="false">$L$14*20</f>
         <v>1033.2</v>
       </c>
-      <c r="M24" s="8" t="n">
+      <c r="M24" s="1" t="n">
         <f aca="false">$M$14*20</f>
         <v>1092.24</v>
       </c>
@@ -2150,19 +2171,19 @@
       <c r="I25" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="J25" s="8" t="n">
+      <c r="J25" s="1" t="n">
         <f aca="false">$J15*20</f>
         <v>623.2</v>
       </c>
-      <c r="K25" s="8" t="n">
+      <c r="K25" s="1" t="n">
         <f aca="false">$K$14*20</f>
         <v>885.6</v>
       </c>
-      <c r="L25" s="8" t="n">
+      <c r="L25" s="1" t="n">
         <f aca="false">$L$14*20</f>
         <v>1033.2</v>
       </c>
-      <c r="M25" s="8" t="n">
+      <c r="M25" s="1" t="n">
         <f aca="false">$M$14*20</f>
         <v>1092.24</v>
       </c>
@@ -2223,19 +2244,19 @@
       <c r="I26" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="J26" s="8" t="n">
+      <c r="J26" s="1" t="n">
         <f aca="false">$J16*20</f>
         <v>656</v>
       </c>
-      <c r="K26" s="8" t="n">
+      <c r="K26" s="1" t="n">
         <f aca="false">$K$14*20</f>
         <v>885.6</v>
       </c>
-      <c r="L26" s="8" t="n">
+      <c r="L26" s="1" t="n">
         <f aca="false">$L$14*20</f>
         <v>1033.2</v>
       </c>
-      <c r="M26" s="8" t="n">
+      <c r="M26" s="1" t="n">
         <f aca="false">$M$14*20</f>
         <v>1092.24</v>
       </c>
@@ -2316,19 +2337,19 @@
       <c r="I28" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="J28" s="8" t="n">
+      <c r="J28" s="1" t="n">
         <f aca="false">J11*21</f>
         <v>516.6</v>
       </c>
-      <c r="K28" s="8" t="n">
+      <c r="K28" s="1" t="n">
         <f aca="false">K11*21</f>
         <v>774.9</v>
       </c>
-      <c r="L28" s="8" t="n">
+      <c r="L28" s="1" t="n">
         <f aca="false">L11*21</f>
         <v>904.05</v>
       </c>
-      <c r="M28" s="8" t="n">
+      <c r="M28" s="1" t="n">
         <f aca="false">M11*21</f>
         <v>955.71</v>
       </c>
@@ -2388,19 +2409,19 @@
       <c r="I29" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="J29" s="8" t="n">
+      <c r="J29" s="1" t="n">
         <f aca="false">J12*21</f>
         <v>551.04</v>
       </c>
-      <c r="K29" s="8" t="n">
+      <c r="K29" s="1" t="n">
         <f aca="false">K12*21</f>
         <v>826.56</v>
       </c>
-      <c r="L29" s="8" t="n">
+      <c r="L29" s="1" t="n">
         <f aca="false">L12*21</f>
         <v>964.32</v>
       </c>
-      <c r="M29" s="8" t="n">
+      <c r="M29" s="1" t="n">
         <f aca="false">M12*21</f>
         <v>1019.424</v>
       </c>
@@ -2460,19 +2481,19 @@
       <c r="I30" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J30" s="8" t="n">
+      <c r="J30" s="1" t="n">
         <f aca="false">J13*21</f>
         <v>585.48</v>
       </c>
-      <c r="K30" s="8" t="n">
+      <c r="K30" s="1" t="n">
         <f aca="false">K13*21</f>
         <v>878.22</v>
       </c>
-      <c r="L30" s="8" t="n">
+      <c r="L30" s="1" t="n">
         <f aca="false">L13*21</f>
         <v>1024.59</v>
       </c>
-      <c r="M30" s="8" t="n">
+      <c r="M30" s="1" t="n">
         <f aca="false">M13*21</f>
         <v>1083.138</v>
       </c>
@@ -2532,19 +2553,19 @@
       <c r="I31" s="19" t="n">
         <v>18</v>
       </c>
-      <c r="J31" s="8" t="n">
+      <c r="J31" s="1" t="n">
         <f aca="false">J14*21</f>
         <v>619.92</v>
       </c>
-      <c r="K31" s="8" t="n">
+      <c r="K31" s="1" t="n">
         <f aca="false">K14*21</f>
         <v>929.88</v>
       </c>
-      <c r="L31" s="8" t="n">
+      <c r="L31" s="1" t="n">
         <f aca="false">L14*21</f>
         <v>1084.86</v>
       </c>
-      <c r="M31" s="8" t="n">
+      <c r="M31" s="1" t="n">
         <f aca="false">M14*21</f>
         <v>1146.852</v>
       </c>
@@ -2604,19 +2625,19 @@
       <c r="I32" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="J32" s="8" t="n">
+      <c r="J32" s="1" t="n">
         <f aca="false">J15*21</f>
         <v>654.36</v>
       </c>
-      <c r="K32" s="8" t="n">
+      <c r="K32" s="1" t="n">
         <f aca="false">K15*21</f>
         <v>981.54</v>
       </c>
-      <c r="L32" s="8" t="n">
+      <c r="L32" s="1" t="n">
         <f aca="false">L15*21</f>
         <v>1145.13</v>
       </c>
-      <c r="M32" s="8" t="n">
+      <c r="M32" s="1" t="n">
         <f aca="false">M15*21</f>
         <v>1210.566</v>
       </c>
@@ -2676,19 +2697,19 @@
       <c r="I33" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="J33" s="8" t="n">
+      <c r="J33" s="1" t="n">
         <f aca="false">J16*21</f>
         <v>688.8</v>
       </c>
-      <c r="K33" s="8" t="n">
+      <c r="K33" s="1" t="n">
         <f aca="false">K16*21</f>
         <v>1033.2</v>
       </c>
-      <c r="L33" s="8" t="n">
+      <c r="L33" s="1" t="n">
         <f aca="false">L16*21</f>
         <v>1205.4</v>
       </c>
-      <c r="M33" s="8" t="n">
+      <c r="M33" s="1" t="n">
         <f aca="false">M16*21</f>
         <v>1274.28</v>
       </c>
@@ -3502,39 +3523,39 @@
   <dimension ref="A1:AK80"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="5.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="8" width="7.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="9.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="8" width="8.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="8" width="14.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="9" style="8" width="11.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="9" style="1" width="11.26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="8" t="n">
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>1.18</v>
       </c>
-      <c r="G2" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" s="8" t="n">
+      <c r="G2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="K2" s="8" t="n">
+      <c r="K2" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="L2" s="8" t="n">
+      <c r="L2" s="1" t="n">
         <v>197</v>
       </c>
-      <c r="O2" s="8" t="n">
+      <c r="O2" s="1" t="n">
         <v>1107</v>
       </c>
-      <c r="Q2" s="8" t="n">
+      <c r="Q2" s="1" t="n">
         <v>1135</v>
       </c>
       <c r="S2" s="23" t="n">
@@ -3546,42 +3567,42 @@
       <c r="AA2" s="23" t="n">
         <v>1429</v>
       </c>
-      <c r="AD2" s="8" t="n">
+      <c r="AD2" s="1" t="n">
         <v>1627</v>
       </c>
-      <c r="AE2" s="8" t="n">
+      <c r="AE2" s="1" t="n">
         <v>1672</v>
       </c>
-      <c r="AG2" s="8" t="n">
+      <c r="AG2" s="1" t="n">
         <v>1721</v>
       </c>
-      <c r="AH2" s="8" t="n">
+      <c r="AH2" s="1" t="n">
         <v>1768</v>
       </c>
-      <c r="AI2" s="8" t="n">
+      <c r="AI2" s="1" t="n">
         <v>1865</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="8" t="n">
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1" t="n">
         <v>0.18</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="1" t="n">
         <v>211</v>
       </c>
       <c r="J3" s="23" t="n">
         <v>244</v>
       </c>
-      <c r="K3" s="8" t="n">
+      <c r="K3" s="1" t="n">
         <v>218</v>
       </c>
-      <c r="L3" s="8" t="n">
+      <c r="L3" s="1" t="n">
         <v>278</v>
       </c>
       <c r="O3" s="23" t="n">
@@ -3602,60 +3623,60 @@
       <c r="AA3" s="23" t="n">
         <v>194</v>
       </c>
-      <c r="AD3" s="8" t="n">
+      <c r="AD3" s="1" t="n">
         <v>193</v>
       </c>
-      <c r="AE3" s="8" t="n">
+      <c r="AE3" s="1" t="n">
         <v>193</v>
       </c>
       <c r="AG3" s="23" t="n">
         <v>271</v>
       </c>
-      <c r="AH3" s="8" t="n">
+      <c r="AH3" s="1" t="n">
         <v>177</v>
       </c>
-      <c r="AI3" s="8" t="n">
+      <c r="AI3" s="1" t="n">
         <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G4" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" s="8" t="n">
+      <c r="G4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="J4" s="8" t="n">
+      <c r="J4" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="K4" s="8" t="n">
+      <c r="K4" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="Z4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="AD4" s="8" t="s">
+      <c r="Z4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AG4" s="8" t="s">
+      <c r="AD4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AH4" s="8" t="s">
+      <c r="AG4" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="AH4" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="AC5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="AH5" s="8" t="s">
+      <c r="AC5" s="1" t="s">
         <v>19</v>
+      </c>
+      <c r="AH5" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="24"/>
       <c r="B11" s="24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>3</v>
@@ -3807,7 +3828,7 @@
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="27"/>
       <c r="B14" s="27" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14" s="27"/>
       <c r="D14" s="27"/>
@@ -4131,7 +4152,7 @@
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27"/>
       <c r="B18" s="27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C18" s="34"/>
       <c r="D18" s="34"/>
@@ -4210,7 +4231,7 @@
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="27"/>
       <c r="B19" s="27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C19" s="32"/>
       <c r="D19" s="32"/>
@@ -4289,7 +4310,7 @@
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="27"/>
       <c r="B20" s="27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C20" s="34"/>
       <c r="D20" s="34"/>
@@ -4368,7 +4389,7 @@
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="27"/>
       <c r="B21" s="27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C21" s="32"/>
       <c r="D21" s="32"/>
@@ -4448,7 +4469,7 @@
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="29"/>
       <c r="B23" s="37" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,7 +4477,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C24" s="38" t="n">
         <v>15</v>
@@ -4534,7 +4555,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C26" s="38" t="n">
         <v>15</v>
@@ -4612,7 +4633,7 @@
         <v>3</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C28" s="38" t="n">
         <v>15</v>
@@ -4679,7 +4700,7 @@
       <c r="M29" s="24"/>
       <c r="N29" s="24"/>
       <c r="O29" s="42" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P29" s="24"/>
       <c r="Q29" s="24"/>
@@ -4692,7 +4713,7 @@
         <v>4</v>
       </c>
       <c r="B30" s="27" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C30" s="38" t="n">
         <v>23</v>
@@ -4760,7 +4781,7 @@
       <c r="N31" s="24"/>
       <c r="O31" s="24"/>
       <c r="P31" s="24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Q31" s="24"/>
       <c r="R31" s="24"/>
@@ -4772,7 +4793,7 @@
         <v>5</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C32" s="38" t="n">
         <v>15</v>
@@ -4850,7 +4871,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="27" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C34" s="38" t="n">
         <v>18</v>
@@ -4928,7 +4949,7 @@
         <v>7</v>
       </c>
       <c r="B36" s="27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C36" s="38" t="n">
         <v>14</v>
@@ -4993,7 +5014,7 @@
       <c r="K37" s="24"/>
       <c r="L37" s="24"/>
       <c r="M37" s="24" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N37" s="24"/>
       <c r="O37" s="24"/>
@@ -5008,7 +5029,7 @@
         <v>8</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C38" s="38" t="n">
         <v>18</v>
@@ -5086,7 +5107,7 @@
         <v>9</v>
       </c>
       <c r="B40" s="27" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C40" s="38" t="n">
         <v>12</v>
@@ -5151,7 +5172,7 @@
       <c r="K41" s="24"/>
       <c r="L41" s="24"/>
       <c r="M41" s="24" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N41" s="24"/>
       <c r="O41" s="24"/>
@@ -5166,7 +5187,7 @@
         <v>10</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C42" s="38" t="n">
         <v>15</v>
@@ -5235,16 +5256,16 @@
       <c r="O43" s="24"/>
       <c r="P43" s="24"/>
       <c r="Q43" s="24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="R43" s="24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S43" s="24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T43" s="24" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5252,7 +5273,7 @@
         <v>11</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C44" s="38" t="n">
         <v>15</v>
@@ -5330,7 +5351,7 @@
         <v>12</v>
       </c>
       <c r="B46" s="27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C46" s="38" t="n">
         <v>15</v>
@@ -5408,7 +5429,7 @@
         <v>13</v>
       </c>
       <c r="B48" s="27" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C48" s="38" t="n">
         <v>19</v>
@@ -5486,7 +5507,7 @@
         <v>14</v>
       </c>
       <c r="B50" s="45" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C50" s="46" t="n">
         <v>21</v>
@@ -5504,32 +5525,32 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="8" t="s">
-        <v>45</v>
+      <c r="B51" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="D51" s="48"/>
       <c r="E51" s="48"/>
-      <c r="J51" s="8" t="s">
-        <v>46</v>
+      <c r="J51" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="R51" s="49" t="s">
-        <v>46</v>
-      </c>
-      <c r="S51" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="U51" s="8" t="s">
         <v>47</v>
       </c>
+      <c r="S51" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="U51" s="1" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F52" s="8"/>
-      <c r="AK52" s="8"/>
+      <c r="F52" s="1"/>
+      <c r="AK52" s="1"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="24"/>
       <c r="B53" s="24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C53" s="24" t="n">
         <v>10</v>
@@ -5615,13 +5636,13 @@
       <c r="AK54" s="24"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F55" s="8"/>
-      <c r="AK55" s="8"/>
+      <c r="F55" s="1"/>
+      <c r="AK55" s="1"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="27"/>
       <c r="B56" s="27" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C56" s="27"/>
       <c r="D56" s="27"/>
@@ -5765,7 +5786,7 @@
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="27"/>
       <c r="B58" s="27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C58" s="34"/>
       <c r="D58" s="34"/>
@@ -5902,7 +5923,7 @@
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="27"/>
       <c r="B59" s="27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C59" s="32"/>
       <c r="D59" s="32"/>
@@ -6039,7 +6060,7 @@
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="27"/>
       <c r="B60" s="27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C60" s="34"/>
       <c r="D60" s="34"/>
@@ -6176,7 +6197,7 @@
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="27"/>
       <c r="B61" s="27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C61" s="32"/>
       <c r="D61" s="32"/>
@@ -6352,17 +6373,17 @@
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="29"/>
       <c r="B63" s="37" t="s">
-        <v>26</v>
-      </c>
-      <c r="F63" s="8"/>
-      <c r="AK63" s="8"/>
+        <v>27</v>
+      </c>
+      <c r="F63" s="1"/>
+      <c r="AK63" s="1"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="29" t="n">
         <v>1</v>
       </c>
       <c r="B64" s="27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C64" s="38" t="n">
         <v>15</v>
@@ -6477,7 +6498,7 @@
         <v>2</v>
       </c>
       <c r="B65" s="27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C65" s="38" t="n">
         <v>15</v>
@@ -6592,7 +6613,7 @@
         <v>3</v>
       </c>
       <c r="B66" s="27" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C66" s="38" t="n">
         <v>15</v>
@@ -6707,7 +6728,7 @@
         <v>4</v>
       </c>
       <c r="B67" s="27" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C67" s="38" t="n">
         <v>23</v>
@@ -6758,7 +6779,7 @@
         <v>5</v>
       </c>
       <c r="B68" s="27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C68" s="38" t="n">
         <v>15</v>
@@ -6873,7 +6894,7 @@
         <v>6</v>
       </c>
       <c r="B69" s="27" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C69" s="38" t="n">
         <v>18</v>
@@ -6988,7 +7009,7 @@
         <v>7</v>
       </c>
       <c r="B70" s="27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C70" s="38" t="n">
         <v>14</v>
@@ -7103,7 +7124,7 @@
         <v>8</v>
       </c>
       <c r="B71" s="27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C71" s="38" t="n">
         <v>18</v>
@@ -7218,7 +7239,7 @@
         <v>9</v>
       </c>
       <c r="B72" s="27" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C72" s="38" t="n">
         <v>18</v>
@@ -7333,7 +7354,7 @@
         <v>10</v>
       </c>
       <c r="B73" s="27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C73" s="38" t="n">
         <v>15</v>
@@ -7448,7 +7469,7 @@
         <v>11</v>
       </c>
       <c r="B74" s="27" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C74" s="38" t="n">
         <v>15</v>
@@ -7563,7 +7584,7 @@
         <v>12</v>
       </c>
       <c r="B75" s="27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C75" s="38" t="n">
         <v>15</v>
@@ -7678,7 +7699,7 @@
         <v>13</v>
       </c>
       <c r="B76" s="27" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C76" s="38" t="n">
         <v>19</v>
@@ -7793,7 +7814,7 @@
         <v>14</v>
       </c>
       <c r="B77" s="45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C77" s="50" t="n">
         <v>21</v>
@@ -7908,7 +7929,7 @@
         <v>14</v>
       </c>
       <c r="B78" s="45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C78" s="50" t="n">
         <v>21</v>
@@ -8023,7 +8044,7 @@
         <v>15</v>
       </c>
       <c r="B79" s="45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C79" s="50" t="n">
         <v>21</v>
@@ -8138,7 +8159,7 @@
         <v>15</v>
       </c>
       <c r="B80" s="45" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C80" s="50" t="n">
         <v>21</v>
@@ -8267,46 +8288,46 @@
   <dimension ref="A1:AK36"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="5.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="8" width="7.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="9.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="8" width="8.62"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="8" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="8" width="14.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="10" style="8" width="11.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.62"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="10" style="1" width="11.26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" s="8" t="n">
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" s="1" t="n">
         <v>83</v>
       </c>
-      <c r="G1" s="8" t="n">
+      <c r="G1" s="1" t="n">
         <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="8" t="n">
+      <c r="B2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="1" t="n">
         <v>1865</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="1" t="n">
         <v>1865</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="1" t="n">
         <v>65</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="1" t="n">
         <v>68</v>
       </c>
       <c r="H3" s="23" t="n">
@@ -8314,42 +8335,42 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="8" t="n">
+      <c r="B4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="1" t="n">
         <v>17</v>
       </c>
       <c r="G4" s="53" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G5" s="8" t="s">
-        <v>53</v>
+      <c r="G5" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="8" t="n">
+      <c r="B7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>1.18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="8" t="n">
+      <c r="B8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="1" t="n">
         <v>0.18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24"/>
       <c r="B10" s="24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="24" t="n">
         <v>10</v>
@@ -8435,8 +8456,8 @@
       <c r="AK11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F12" s="8" t="s">
-        <v>54</v>
+      <c r="F12" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8584,7 +8605,7 @@
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27"/>
       <c r="B15" s="27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C15" s="34"/>
       <c r="D15" s="34"/>
@@ -8628,7 +8649,7 @@
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27"/>
       <c r="B16" s="27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C16" s="32"/>
       <c r="D16" s="32"/>
@@ -8672,7 +8693,7 @@
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="27"/>
       <c r="B17" s="27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17" s="34"/>
       <c r="D17" s="34"/>
@@ -8716,7 +8737,7 @@
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27"/>
       <c r="B18" s="27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C18" s="32"/>
       <c r="D18" s="32"/>
@@ -8799,7 +8820,7 @@
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29"/>
       <c r="B20" s="37" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8807,7 +8828,7 @@
         <v>1</v>
       </c>
       <c r="B21" s="27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C21" s="38" t="n">
         <v>15</v>
@@ -8831,7 +8852,7 @@
         <v>2</v>
       </c>
       <c r="B22" s="27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="38" t="n">
         <v>15</v>
@@ -8855,7 +8876,7 @@
         <v>3</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C23" s="38" t="n">
         <v>15</v>
@@ -8879,7 +8900,7 @@
         <v>4</v>
       </c>
       <c r="B24" s="27" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C24" s="38" t="n">
         <v>23</v>
@@ -8901,7 +8922,7 @@
         <v>5</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C25" s="38" t="n">
         <v>15</v>
@@ -8925,7 +8946,7 @@
         <v>6</v>
       </c>
       <c r="B26" s="27" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C26" s="38" t="n">
         <v>18</v>
@@ -8949,7 +8970,7 @@
         <v>7</v>
       </c>
       <c r="B27" s="27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C27" s="38" t="n">
         <v>14</v>
@@ -8973,7 +8994,7 @@
         <v>8</v>
       </c>
       <c r="B28" s="27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28" s="38" t="n">
         <v>18</v>
@@ -8997,7 +9018,7 @@
         <v>9</v>
       </c>
       <c r="B29" s="27" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C29" s="38" t="n">
         <v>18</v>
@@ -9021,7 +9042,7 @@
         <v>10</v>
       </c>
       <c r="B30" s="27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C30" s="38" t="n">
         <v>15</v>
@@ -9045,7 +9066,7 @@
         <v>11</v>
       </c>
       <c r="B31" s="27" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C31" s="38" t="n">
         <v>15</v>
@@ -9069,7 +9090,7 @@
         <v>12</v>
       </c>
       <c r="B32" s="27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C32" s="38" t="n">
         <v>15</v>
@@ -9093,7 +9114,7 @@
         <v>13</v>
       </c>
       <c r="B33" s="27" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C33" s="38" t="n">
         <v>19</v>
@@ -9117,7 +9138,7 @@
         <v>14</v>
       </c>
       <c r="B34" s="45" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C34" s="46" t="n">
         <v>21</v>
@@ -9138,7 +9159,7 @@
       <c r="F35" s="48"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J36" s="8" t="n">
+      <c r="J36" s="1" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WhiteBoard Update - 2026-05-04 10:36:07
</commit_message>
<xml_diff>
--- a/MyPreply/PreplyAnalyse-2.xlsx
+++ b/MyPreply/PreplyAnalyse-2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Ranking" sheetId="1" state="visible" r:id="rId3"/>
@@ -8379,7 +8379,7 @@
       <c r="E10" s="24"/>
       <c r="F10" s="25" t="n">
         <f aca="false">F$17*$C$10+F$15</f>
-        <v>991.357926221336</v>
+        <v>869.327001753361</v>
       </c>
       <c r="G10" s="24"/>
       <c r="H10" s="24"/>
@@ -8421,7 +8421,7 @@
       <c r="E11" s="24"/>
       <c r="F11" s="25" t="n">
         <f aca="false">F10/$C$7</f>
-        <v>840.133835780793</v>
+        <v>736.717798096069</v>
       </c>
       <c r="G11" s="24"/>
       <c r="H11" s="24"/>
@@ -8612,7 +8612,7 @@
       <c r="E15" s="34"/>
       <c r="F15" s="35" t="n">
         <f aca="false">SUMPRODUCT(F$21:F$33,$C$21:$C$33)*(1-$C$8)</f>
-        <v>881.5</v>
+        <v>758.5</v>
       </c>
       <c r="G15" s="34"/>
       <c r="H15" s="34"/>
@@ -8656,7 +8656,7 @@
       <c r="E16" s="32"/>
       <c r="F16" s="36" t="n">
         <f aca="false">F$15/$C$7</f>
-        <v>747.033898305085</v>
+        <v>642.796610169492</v>
       </c>
       <c r="G16" s="32"/>
       <c r="H16" s="32"/>
@@ -8700,7 +8700,7 @@
       <c r="E17" s="34"/>
       <c r="F17" s="35" t="n">
         <f aca="false">F$16/(SUM(F$21:F$33))</f>
-        <v>10.9857926221336</v>
+        <v>11.0827001753361</v>
       </c>
       <c r="G17" s="34"/>
       <c r="H17" s="34"/>
@@ -8744,7 +8744,7 @@
       <c r="E18" s="32"/>
       <c r="F18" s="36" t="n">
         <f aca="false">F$17/$C$7</f>
-        <v>9.30999374757085</v>
+        <v>9.39211879265768</v>
       </c>
       <c r="G18" s="32"/>
       <c r="H18" s="32"/>
@@ -8890,7 +8890,7 @@
         <v>10.4237288135593</v>
       </c>
       <c r="F23" s="24" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I23" s="24"/>
       <c r="J23" s="24"/>

</xml_diff>